<commit_message>
Optimized the endschiessen module and added a new module for sektionrang. The endschiessen module now includes a new file for price logic, and the sektionrang module has several new files for generating PDFs and loading data. Additionally, there are new migration files for updating the database schema and navigation for the sektionrang feature.
</commit_message>
<xml_diff>
--- a/inc/endschloesen/Vorlage/Standblatt_Endschiessen_Vorlage.xlsx
+++ b/inc/endschloesen/Vorlage/Standblatt_Endschiessen_Vorlage.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TEMP\msvjm\msvdev\inc\endschloesen\Vorlage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF46BC77-2538-4B91-8377-31FD0662D2CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D855A3E6-AD70-44AF-8031-3998372BEF57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Tabelle1!$A$1:$Q$75</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Tabelle1!$A$1:$Q$73</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="83">
   <si>
     <t>Zabigstich</t>
   </si>
@@ -295,6 +295,9 @@
   </si>
   <si>
     <t>${sieergeloest}</t>
+  </si>
+  <si>
+    <t>${schwini2geloest}</t>
   </si>
 </sst>
 </file>
@@ -568,7 +571,22 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
@@ -589,28 +607,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1953,7 +1956,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U77"/>
+  <dimension ref="A1:U74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="11.42578125" customWidth="1"/>
@@ -1988,15 +1991,15 @@
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1">
-      <c r="F2" s="35"/>
-      <c r="G2" s="36"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" customHeight="1">
       <c r="A3" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="37"/>
-      <c r="G3" s="38"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="43"/>
       <c r="I3" t="s">
         <v>1</v>
       </c>
@@ -2005,15 +2008,15 @@
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="37"/>
-      <c r="G4" s="38"/>
+      <c r="F4" s="42"/>
+      <c r="G4" s="43"/>
       <c r="I4" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" customHeight="1">
-      <c r="F5" s="37"/>
-      <c r="G5" s="38"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="43"/>
       <c r="I5" t="s">
         <v>69</v>
       </c>
@@ -2022,22 +2025,22 @@
       <c r="A6" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="43" t="s">
+      <c r="B6" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="38"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="F6" s="42"/>
+      <c r="G6" s="43"/>
     </row>
     <row r="7" spans="1:13" ht="15.75" customHeight="1">
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="38"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="43"/>
       <c r="I7" s="6" t="s">
         <v>3</v>
       </c>
@@ -2052,13 +2055,13 @@
       </c>
     </row>
     <row r="8" spans="1:13" ht="15.75" customHeight="1">
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="38"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="43"/>
       <c r="I8" t="s">
         <v>25</v>
       </c>
@@ -2076,15 +2079,15 @@
       <c r="A9" s="6"/>
       <c r="B9" s="7"/>
       <c r="C9" s="1"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="38"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="43"/>
     </row>
     <row r="10" spans="1:13" ht="15.75" customHeight="1">
       <c r="A10" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="F10" s="37"/>
-      <c r="G10" s="38"/>
+      <c r="F10" s="42"/>
+      <c r="G10" s="43"/>
       <c r="I10" s="25" t="s">
         <v>62</v>
       </c>
@@ -2099,8 +2102,8 @@
       <c r="B11" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="37"/>
-      <c r="G11" s="38"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="43"/>
       <c r="J11" s="22" t="s">
         <v>64</v>
       </c>
@@ -2109,15 +2112,15 @@
       <c r="B12" t="s">
         <v>35</v>
       </c>
-      <c r="F12" s="37"/>
-      <c r="G12" s="38"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="43"/>
       <c r="J12" s="22" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:13">
-      <c r="F13" s="37"/>
-      <c r="G13" s="38"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="43"/>
     </row>
     <row r="14" spans="1:13" ht="15.75">
       <c r="A14" t="s">
@@ -2127,8 +2130,8 @@
         <v>36</v>
       </c>
       <c r="E14" s="5"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="40"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="45"/>
     </row>
     <row r="15" spans="1:13">
       <c r="B15" t="s">
@@ -2136,11 +2139,11 @@
       </c>
     </row>
     <row r="16" spans="1:13" ht="15.75" customHeight="1">
-      <c r="K16" s="41" t="s">
+      <c r="K16" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="L16" s="41"/>
-      <c r="M16" s="41"/>
+      <c r="L16" s="34"/>
+      <c r="M16" s="34"/>
     </row>
     <row r="17" spans="1:21" ht="13.5" thickBot="1">
       <c r="A17" s="9"/>
@@ -2166,21 +2169,21 @@
         <v>76</v>
       </c>
       <c r="F19" s="25" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:21" ht="20.25">
       <c r="A20" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="48" t="s">
+      <c r="C20" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="42"/>
-      <c r="F20" s="42" t="s">
+      <c r="D20" s="39"/>
+      <c r="F20" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="G20" s="42"/>
+      <c r="G20" s="39"/>
       <c r="I20" s="8" t="s">
         <v>46</v>
       </c>
@@ -2189,10 +2192,10 @@
       </c>
     </row>
     <row r="21" spans="1:21">
-      <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="F21" s="35"/>
-      <c r="G21" s="36"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="41"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="41"/>
       <c r="I21" t="s">
         <v>47</v>
       </c>
@@ -2201,10 +2204,10 @@
       <c r="A22" t="s">
         <v>7</v>
       </c>
-      <c r="C22" s="37"/>
-      <c r="D22" s="38"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="38"/>
+      <c r="C22" s="42"/>
+      <c r="D22" s="43"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="43"/>
       <c r="P22" s="12"/>
       <c r="Q22" s="10"/>
     </row>
@@ -2212,10 +2215,10 @@
       <c r="A23" t="s">
         <v>8</v>
       </c>
-      <c r="C23" s="37"/>
-      <c r="D23" s="38"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="38"/>
+      <c r="C23" s="42"/>
+      <c r="D23" s="43"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="43"/>
       <c r="I23" s="6" t="s">
         <v>3</v>
       </c>
@@ -2232,38 +2235,38 @@
       <c r="U23" s="1"/>
     </row>
     <row r="24" spans="1:21" ht="12" customHeight="1" thickBot="1">
-      <c r="C24" s="37"/>
-      <c r="D24" s="38"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="38"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="43"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="43"/>
       <c r="I24" s="9"/>
       <c r="J24" s="9"/>
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9"/>
-      <c r="O24" s="46"/>
-      <c r="P24" s="46"/>
-      <c r="Q24" s="46"/>
+      <c r="O24" s="47"/>
+      <c r="P24" s="47"/>
+      <c r="Q24" s="47"/>
     </row>
     <row r="25" spans="1:21" ht="26.25" customHeight="1" thickTop="1">
-      <c r="A25" s="47" t="s">
+      <c r="A25" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="47"/>
-      <c r="C25" s="37"/>
-      <c r="D25" s="38"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="38"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="43"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="43"/>
     </row>
     <row r="26" spans="1:21" ht="20.25">
       <c r="A26" t="s">
         <v>12</v>
       </c>
-      <c r="C26" s="37"/>
-      <c r="D26" s="38"/>
-      <c r="F26" s="37"/>
-      <c r="G26" s="38"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="43"/>
+      <c r="F26" s="42"/>
+      <c r="G26" s="43"/>
       <c r="I26" s="8" t="s">
         <v>70</v>
       </c>
@@ -2275,10 +2278,10 @@
       <c r="A27" t="s">
         <v>13</v>
       </c>
-      <c r="C27" s="37"/>
-      <c r="D27" s="38"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="38"/>
+      <c r="C27" s="42"/>
+      <c r="D27" s="43"/>
+      <c r="F27" s="42"/>
+      <c r="G27" s="43"/>
       <c r="P27" s="28"/>
       <c r="Q27" s="29"/>
     </row>
@@ -2286,10 +2289,10 @@
       <c r="A28" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="37"/>
-      <c r="D28" s="38"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="38"/>
+      <c r="C28" s="42"/>
+      <c r="D28" s="43"/>
+      <c r="F28" s="42"/>
+      <c r="G28" s="43"/>
       <c r="I28" t="s">
         <v>71</v>
       </c>
@@ -2300,10 +2303,10 @@
       <c r="A29" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="37"/>
-      <c r="D29" s="38"/>
-      <c r="F29" s="37"/>
-      <c r="G29" s="38"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="43"/>
+      <c r="F29" s="42"/>
+      <c r="G29" s="43"/>
       <c r="I29" t="s">
         <v>2</v>
       </c>
@@ -2311,18 +2314,18 @@
       <c r="Q29" s="31"/>
     </row>
     <row r="30" spans="1:21">
-      <c r="C30" s="37"/>
-      <c r="D30" s="38"/>
-      <c r="F30" s="37"/>
-      <c r="G30" s="38"/>
+      <c r="C30" s="42"/>
+      <c r="D30" s="43"/>
+      <c r="F30" s="42"/>
+      <c r="G30" s="43"/>
       <c r="P30" s="30"/>
       <c r="Q30" s="31"/>
     </row>
     <row r="31" spans="1:21">
-      <c r="C31" s="37"/>
-      <c r="D31" s="38"/>
-      <c r="F31" s="37"/>
-      <c r="G31" s="38"/>
+      <c r="C31" s="42"/>
+      <c r="D31" s="43"/>
+      <c r="F31" s="42"/>
+      <c r="G31" s="43"/>
       <c r="I31" s="6" t="s">
         <v>3</v>
       </c>
@@ -2339,18 +2342,18 @@
       <c r="Q31" s="31"/>
     </row>
     <row r="32" spans="1:21">
-      <c r="C32" s="37"/>
-      <c r="D32" s="38"/>
-      <c r="F32" s="37"/>
-      <c r="G32" s="38"/>
+      <c r="C32" s="42"/>
+      <c r="D32" s="43"/>
+      <c r="F32" s="42"/>
+      <c r="G32" s="43"/>
       <c r="P32" s="30"/>
       <c r="Q32" s="31"/>
     </row>
     <row r="33" spans="1:17" ht="20.25" customHeight="1">
-      <c r="C33" s="39"/>
-      <c r="D33" s="40"/>
-      <c r="F33" s="39"/>
-      <c r="G33" s="40"/>
+      <c r="C33" s="44"/>
+      <c r="D33" s="45"/>
+      <c r="F33" s="44"/>
+      <c r="G33" s="45"/>
       <c r="P33" s="30"/>
       <c r="Q33" s="31"/>
     </row>
@@ -2435,26 +2438,26 @@
       </c>
     </row>
     <row r="43" spans="1:17" ht="15.75" customHeight="1">
-      <c r="F43" s="35"/>
-      <c r="G43" s="36"/>
+      <c r="F43" s="40"/>
+      <c r="G43" s="41"/>
     </row>
     <row r="44" spans="1:17" ht="15.75" customHeight="1">
       <c r="A44" t="s">
         <v>26</v>
       </c>
-      <c r="F44" s="37"/>
-      <c r="G44" s="38"/>
+      <c r="F44" s="42"/>
+      <c r="G44" s="43"/>
     </row>
     <row r="45" spans="1:17" ht="15.75" customHeight="1">
       <c r="A45" t="s">
         <v>2</v>
       </c>
-      <c r="F45" s="37"/>
-      <c r="G45" s="38"/>
+      <c r="F45" s="42"/>
+      <c r="G45" s="43"/>
     </row>
     <row r="46" spans="1:17" ht="15.75" customHeight="1">
-      <c r="F46" s="37"/>
-      <c r="G46" s="38"/>
+      <c r="F46" s="42"/>
+      <c r="G46" s="43"/>
     </row>
     <row r="47" spans="1:17" ht="15.75" customHeight="1">
       <c r="A47" s="6" t="s">
@@ -2468,8 +2471,8 @@
       </c>
       <c r="D47" s="24"/>
       <c r="E47" s="24"/>
-      <c r="F47" s="37"/>
-      <c r="G47" s="38"/>
+      <c r="F47" s="42"/>
+      <c r="G47" s="43"/>
       <c r="I47" s="15"/>
       <c r="J47" s="15"/>
       <c r="K47" s="15"/>
@@ -2481,31 +2484,31 @@
       <c r="Q47" s="15"/>
     </row>
     <row r="48" spans="1:17" ht="15.75" customHeight="1">
-      <c r="C48" s="43" t="s">
+      <c r="C48" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="D48" s="44"/>
-      <c r="E48" s="45"/>
-      <c r="F48" s="37"/>
-      <c r="G48" s="38"/>
+      <c r="D48" s="36"/>
+      <c r="E48" s="46"/>
+      <c r="F48" s="42"/>
+      <c r="G48" s="43"/>
     </row>
     <row r="49" spans="1:17" ht="15.75" customHeight="1">
       <c r="C49" t="s">
         <v>23</v>
       </c>
-      <c r="F49" s="37"/>
-      <c r="G49" s="38"/>
+      <c r="F49" s="42"/>
+      <c r="G49" s="43"/>
     </row>
     <row r="50" spans="1:17" ht="15.75" customHeight="1">
-      <c r="F50" s="37"/>
-      <c r="G50" s="38"/>
+      <c r="F50" s="42"/>
+      <c r="G50" s="43"/>
     </row>
     <row r="51" spans="1:17" ht="15.75" customHeight="1">
       <c r="A51" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="F51" s="37"/>
-      <c r="G51" s="38"/>
+      <c r="F51" s="42"/>
+      <c r="G51" s="43"/>
     </row>
     <row r="52" spans="1:17" ht="15.75" customHeight="1">
       <c r="A52" t="s">
@@ -2514,8 +2517,8 @@
       <c r="B52" t="s">
         <v>39</v>
       </c>
-      <c r="F52" s="39"/>
-      <c r="G52" s="40"/>
+      <c r="F52" s="44"/>
+      <c r="G52" s="45"/>
     </row>
     <row r="53" spans="1:17">
       <c r="B53" t="s">
@@ -2572,26 +2575,26 @@
       <c r="A63" t="s">
         <v>28</v>
       </c>
-      <c r="F63" s="35"/>
-      <c r="G63" s="36"/>
-      <c r="I63" s="34"/>
-      <c r="J63" s="34"/>
-      <c r="L63" s="41"/>
-      <c r="M63" s="41"/>
-      <c r="N63" s="41"/>
-      <c r="O63" s="41"/>
-      <c r="P63" s="41"/>
+      <c r="F63" s="40"/>
+      <c r="G63" s="41"/>
+      <c r="I63" s="48"/>
+      <c r="J63" s="48"/>
+      <c r="L63" s="34"/>
+      <c r="M63" s="34"/>
+      <c r="N63" s="34"/>
+      <c r="O63" s="34"/>
+      <c r="P63" s="34"/>
     </row>
     <row r="64" spans="1:17" ht="15.75" customHeight="1">
       <c r="A64" t="s">
         <v>2</v>
       </c>
-      <c r="F64" s="37"/>
-      <c r="G64" s="38"/>
-      <c r="I64" s="34" t="s">
+      <c r="F64" s="42"/>
+      <c r="G64" s="43"/>
+      <c r="I64" s="48" t="s">
         <v>60</v>
       </c>
-      <c r="J64" s="34"/>
+      <c r="J64" s="48"/>
       <c r="L64" s="27" t="s">
         <v>73</v>
       </c>
@@ -2601,31 +2604,31 @@
       <c r="P64" s="27"/>
     </row>
     <row r="65" spans="1:17" ht="15.75" customHeight="1">
-      <c r="F65" s="37"/>
-      <c r="G65" s="38"/>
-      <c r="L65" s="41"/>
-      <c r="M65" s="41"/>
-      <c r="N65" s="41"/>
-      <c r="O65" s="41"/>
-      <c r="P65" s="41"/>
+      <c r="F65" s="42"/>
+      <c r="G65" s="43"/>
+      <c r="L65" s="34"/>
+      <c r="M65" s="34"/>
+      <c r="N65" s="34"/>
+      <c r="O65" s="34"/>
+      <c r="P65" s="34"/>
     </row>
     <row r="66" spans="1:17" ht="15.75" customHeight="1">
       <c r="A66" t="s">
         <v>10</v>
       </c>
-      <c r="F66" s="37"/>
-      <c r="G66" s="38"/>
-      <c r="I66" s="34" t="s">
+      <c r="F66" s="42"/>
+      <c r="G66" s="43"/>
+      <c r="I66" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="J66" s="34"/>
+      <c r="J66" s="48"/>
     </row>
     <row r="67" spans="1:17" ht="15.75" customHeight="1">
       <c r="A67" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F67" s="37"/>
-      <c r="G67" s="38"/>
+      <c r="F67" s="42"/>
+      <c r="G67" s="43"/>
       <c r="I67" s="26"/>
       <c r="J67" s="26"/>
       <c r="L67" s="21"/>
@@ -2641,8 +2644,11 @@
       <c r="B68" t="s">
         <v>14</v>
       </c>
-      <c r="F68" s="39"/>
-      <c r="G68" s="40"/>
+      <c r="F68" s="44"/>
+      <c r="G68" s="45"/>
+      <c r="L68" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="69" spans="1:17" ht="15.75" customHeight="1">
       <c r="A69" s="1" t="s">
@@ -2651,79 +2657,68 @@
       <c r="B69" t="s">
         <v>16</v>
       </c>
-      <c r="L69" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="72" spans="1:17" ht="13.5" thickBot="1">
-      <c r="A72" s="6" t="s">
+    </row>
+    <row r="70" spans="1:17" ht="13.5" thickBot="1"/>
+    <row r="71" spans="1:17">
+      <c r="A71" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B72" s="7" t="s">
+      <c r="B71" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C72" s="1" t="s">
+      <c r="C71" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D72" t="s">
+      <c r="D71" t="s">
         <v>5</v>
       </c>
+      <c r="G71" s="2"/>
+      <c r="I71" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="J71" s="26"/>
+      <c r="L71" s="2"/>
+      <c r="N71" s="2"/>
+      <c r="P71" s="2"/>
+    </row>
+    <row r="72" spans="1:17" ht="17.25" customHeight="1" thickBot="1">
+      <c r="D72" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G72" s="3"/>
+      <c r="I72" s="26"/>
+      <c r="J72" s="26"/>
+      <c r="L72" s="4"/>
+      <c r="N72" s="4"/>
+      <c r="P72" s="4"/>
     </row>
     <row r="73" spans="1:17" ht="13.5" thickBot="1">
-      <c r="G73" s="2"/>
-      <c r="I73" s="26"/>
-      <c r="J73" s="26"/>
-    </row>
-    <row r="74" spans="1:17" ht="17.25" customHeight="1">
-      <c r="D74" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="G74" s="3"/>
-      <c r="I74" s="34" t="s">
-        <v>59</v>
-      </c>
-      <c r="J74" s="34"/>
-      <c r="L74" s="2"/>
-      <c r="N74" s="2"/>
-      <c r="P74" s="2"/>
-    </row>
-    <row r="75" spans="1:17" ht="13.5" thickBot="1">
-      <c r="G75" s="4"/>
-      <c r="I75" s="34"/>
-      <c r="J75" s="34"/>
-      <c r="L75" s="4"/>
-      <c r="N75" s="4"/>
-      <c r="P75" s="4"/>
-      <c r="Q75" s="18"/>
-    </row>
-    <row r="76" spans="1:17">
-      <c r="L76" s="19" t="s">
+      <c r="G73" s="4"/>
+      <c r="L73" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="M76" s="14"/>
-      <c r="N76" s="19" t="s">
+      <c r="M73" s="14"/>
+      <c r="N73" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="O76" s="19"/>
-      <c r="P76" s="19" t="s">
+      <c r="O73" s="19"/>
+      <c r="P73" s="19" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="77" spans="1:17">
-      <c r="N77" s="14" t="s">
+      <c r="Q73" s="18"/>
+    </row>
+    <row r="74" spans="1:17">
+      <c r="N74" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="O77" s="14"/>
+      <c r="O74" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="K16:M16"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D33"/>
+  <mergeCells count="19">
+    <mergeCell ref="I63:J63"/>
+    <mergeCell ref="I64:J64"/>
+    <mergeCell ref="I66:J66"/>
+    <mergeCell ref="F2:G14"/>
     <mergeCell ref="L63:P63"/>
     <mergeCell ref="L65:P65"/>
     <mergeCell ref="F20:G20"/>
@@ -2732,11 +2727,13 @@
     <mergeCell ref="F43:G52"/>
     <mergeCell ref="F21:G33"/>
     <mergeCell ref="O24:Q24"/>
-    <mergeCell ref="I74:J75"/>
-    <mergeCell ref="I63:J63"/>
-    <mergeCell ref="I64:J64"/>
-    <mergeCell ref="I66:J66"/>
-    <mergeCell ref="F2:G14"/>
+    <mergeCell ref="K16:M16"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D33"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.25" right="0.49" top="0.25" bottom="0" header="0" footer="0.08"/>

</xml_diff>